<commit_message>
Bump version to 0.1.17; fix critical shared-strings reader bug, add parallel sheet parsing, expand formula engine with 14 functions + named ranges + array formulas + logic functions, fix formula-cell value leakage, migrate tests to tempfile, regenerate corrupt fixtures, and update documentation
Update version headers and last-updated timestamps to 2026-09-08 across ARCHITECTURE.md, Cargo.toml (0.1.17, rust-version 1.85), README.md, SPEC.md, and TODO.md. Archive XLS_VALIDATION_SUMMARY.md (references
</commit_message>
<xml_diff>
--- a/examples/employees.xlsx
+++ b/examples/employees.xlsx
@@ -15,38 +15,25 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
+      <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
-      <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF4472C4"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FFEFEFEF"/>
+        <bgColor rgb="FFEFEFEF"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -54,38 +41,16 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
 </file>
 
@@ -204,7 +169,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -223,14 +188,19 @@
           <t>Department</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Alice</t>
+          <t>Alice Johnson</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -238,20 +208,98 @@
           <t>Engineering</t>
         </is>
       </c>
+      <c r="D2">
+        <v>85000</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Bob</t>
+          <t>Bob Smith</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
+      </c>
+      <c r="D3">
+        <v>65000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Carol Davis</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D4">
+        <v>92000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Dan Miller</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="D5">
+        <v>72000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>6</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Grace Anderson</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D6">
+        <v>81000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>7</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Henry Wilson</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D7">
+        <v>95000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>